<commit_message>
Nuevos test cases incorporados
</commit_message>
<xml_diff>
--- a/Modelo Test Plan.xlsx
+++ b/Modelo Test Plan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiro\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiro\CoderBits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A10628A-562C-48EE-8AD4-FB94922E0CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A6B122-C029-40E8-8A25-C4A60EDDFED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{96765352-7388-4C61-94B8-5077301D3254}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="120">
   <si>
     <t>MODULOS</t>
   </si>
@@ -183,12 +183,6 @@
   </si>
   <si>
     <t xml:space="preserve">  "detail": "Credenciales incorrectas"</t>
-  </si>
-  <si>
-    <t>Validacion de campos</t>
-  </si>
-  <si>
-    <t>Edgar Pena</t>
   </si>
   <si>
     <t>Status: 201 Created</t>
@@ -338,12 +332,6 @@
     <t>El sistema debe eliminar al personal de manera logica y poder recuperarlo luego</t>
   </si>
   <si>
-    <t>Status: 200 OK</t>
-  </si>
-  <si>
-    <t>Status: 204 No Content</t>
-  </si>
-  <si>
     <t>Recuperacion de personal eliminado</t>
   </si>
   <si>
@@ -422,13 +410,89 @@
   </si>
   <si>
     <t>Conexión al websocke de alertar ws://127.0.0.1:8000/ws/alertas/</t>
+  </si>
+  <si>
+    <t>https://github.com/alejav0240/CoderBits/issues/32</t>
+  </si>
+  <si>
+    <t>Usuario eliminado logicamente</t>
+  </si>
+  <si>
+    <t>Creacion de mitigacion según el ataque</t>
+  </si>
+  <si>
+    <t>El sistema tiene que generar su mitigacion correspondiente a cada registro de ataque que se genere</t>
+  </si>
+  <si>
+    <t>Mitigacion creada respecto a la ip del atacante</t>
+  </si>
+  <si>
+    <t>Envio de los datos en tiempo real</t>
+  </si>
+  <si>
+    <t>El sistema debe mandar los datos atravez del websocket en tiempo real</t>
+  </si>
+  <si>
+    <t>"tipo_evento": "conexion",
+    "conexion": {
+        "ip_src": "47.90.134.154",
+        "ip_dst": "192.168.0.35",
+        "port_dst": null,
+        "protocolo": "UDP",
+        "timestamp": "2025-10-16T02:05:22.998676+00:00"
+    }</t>
+  </si>
+  <si>
+    <t>Hasheo de contraseña</t>
+  </si>
+  <si>
+    <t>El sistema debe hashear la contraseña del usuario</t>
+  </si>
+  <si>
+    <t>Generacion de reportes</t>
+  </si>
+  <si>
+    <t>El sistema debe poder generar reportes con datos recibidos atravez del backend</t>
+  </si>
+  <si>
+    <t>Peticion a: api/dashboard/stats/</t>
+  </si>
+  <si>
+    <t>"ataques_activos": x,
+  "ataques_hoy": x,
+  "conexiones_hoy": x,
+  "mitigaciones_exitosas": x,
+  "ataques_ultimos_30_dias": x</t>
+  </si>
+  <si>
+    <t>Generacion de estadisticas para reportes</t>
+  </si>
+  <si>
+    <t>El sistema debe poder generar reportes estadisticas del dia que se pide el reporte</t>
+  </si>
+  <si>
+    <t>Peticion a: api/dashboard/export/json/</t>
+  </si>
+  <si>
+    <t>"ataques": [
+    {
+      "id": x,
+      "tipo": x,
+      "descripcion": x,
+      "ip_origen": x,
+      "ip_destino":x,
+      "puerto": x,
+      "fecha_detectado": "fecha del dia que se pidio el reporte",
+      "conteo_conexiones": x,
+      "activo": x
+    },.........</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -438,6 +502,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -460,10 +532,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -489,92 +562,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="63">
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -694,6 +690,87 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center"/>
@@ -6562,54 +6639,54 @@
     <dataField name="Cuenta de Estado (Dropdown)" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="14">
-    <format dxfId="43">
+    <format dxfId="16">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="14">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="10">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="9">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="8">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="34">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="4">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -6756,60 +6833,60 @@
     <dataField name="Cuenta de Test Case" fld="1" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="16">
-    <format dxfId="59">
+    <format dxfId="32">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="31">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="57">
+    <format dxfId="30">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="29">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="55">
+    <format dxfId="28">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="54">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="24">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="23">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="22">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="48">
+    <format dxfId="21">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="47">
+    <format dxfId="20">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="46">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="45">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -6919,22 +6996,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{580B5FFA-030D-4D17-8F6D-90DDF4342984}" name="TestPlan" displayName="TestPlan" ref="A2:M140" headerRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{580B5FFA-030D-4D17-8F6D-90DDF4342984}" name="TestPlan" displayName="TestPlan" ref="A2:M140" headerRowDxfId="59">
   <autoFilter ref="A2:M140" xr:uid="{580B5FFA-030D-4D17-8F6D-90DDF4342984}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{7F95280F-E669-4A5D-AEDF-FCAAAC81F275}" name="Modulo (Dropdown)" totalsRowLabel="Total" dataDxfId="24" totalsRowDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{E775B39B-DEB6-4123-A65F-A37EDA4383A3}" name="Test Case" dataDxfId="22" totalsRowDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{4E500E60-0861-4EF2-B610-79885F5EF7FD}" name="Descripción" dataDxfId="20" totalsRowDxfId="21"/>
-    <tableColumn id="14" xr3:uid="{D149BE2F-3E66-4E54-8D0E-BA4D69F73794}" name="Tipo/s de Prueba" dataDxfId="18" totalsRowDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{48166857-FFB0-4E91-A69A-8A057DEBB914}" name="Precondiciones" dataDxfId="16" totalsRowDxfId="17"/>
-    <tableColumn id="13" xr3:uid="{09440620-A437-484D-9292-769D8C979710}" name="Pasos a seguir" dataDxfId="14" totalsRowDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{25FFAFC4-E636-4C78-8EC4-9B105CD6EC6A}" name="Datos de Prueba" dataDxfId="12" totalsRowDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{5C319188-663F-4BD1-ADB0-A93CF2F134F5}" name="Resultado Esperado" dataDxfId="10" totalsRowDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{AC65C1EE-D520-403E-8171-F3B42F898A90}" name="Resultado Actual (Si falla)" dataDxfId="8" totalsRowDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{67BFFC43-BD7A-400D-BCA5-7641851369E7}" name="Ultima ejecución (Fecha)" dataDxfId="6" totalsRowDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{AF2F4479-94ED-46CC-8F6A-9945904E34B4}" name="Encargado de Prueba" dataDxfId="4" totalsRowDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{1AE568CA-11EA-494D-A158-098CEC0427F1}" name="Estado (Dropdown)" dataDxfId="2" totalsRowDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{D7CC1236-1B17-4FEE-A062-7A6AF5789012}" name="Comentario" totalsRowFunction="count" dataDxfId="0" totalsRowDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{7F95280F-E669-4A5D-AEDF-FCAAAC81F275}" name="Modulo (Dropdown)" totalsRowLabel="Total" dataDxfId="58" totalsRowDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{E775B39B-DEB6-4123-A65F-A37EDA4383A3}" name="Test Case" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{4E500E60-0861-4EF2-B610-79885F5EF7FD}" name="Descripción" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="14" xr3:uid="{D149BE2F-3E66-4E54-8D0E-BA4D69F73794}" name="Tipo/s de Prueba" dataDxfId="52" totalsRowDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{48166857-FFB0-4E91-A69A-8A057DEBB914}" name="Precondiciones" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="13" xr3:uid="{09440620-A437-484D-9292-769D8C979710}" name="Pasos a seguir" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="12" xr3:uid="{25FFAFC4-E636-4C78-8EC4-9B105CD6EC6A}" name="Datos de Prueba" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{5C319188-663F-4BD1-ADB0-A93CF2F134F5}" name="Resultado Esperado" dataDxfId="44" totalsRowDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{AC65C1EE-D520-403E-8171-F3B42F898A90}" name="Resultado Actual (Si falla)" dataDxfId="42" totalsRowDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{67BFFC43-BD7A-400D-BCA5-7641851369E7}" name="Ultima ejecución (Fecha)" dataDxfId="40" totalsRowDxfId="39"/>
+    <tableColumn id="10" xr3:uid="{AF2F4479-94ED-46CC-8F6A-9945904E34B4}" name="Encargado de Prueba" dataDxfId="38" totalsRowDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{1AE568CA-11EA-494D-A158-098CEC0427F1}" name="Estado (Dropdown)" dataDxfId="36" totalsRowDxfId="35"/>
+    <tableColumn id="9" xr3:uid="{D7CC1236-1B17-4FEE-A062-7A6AF5789012}" name="Comentario" totalsRowFunction="count" dataDxfId="34" totalsRowDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7452,7 +7529,9 @@
       <c r="D4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="7"/>
+      <c r="E4" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="F4" s="7" t="s">
         <v>43</v>
       </c>
@@ -7474,38 +7553,52 @@
       </c>
       <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
       <c r="I5" s="7"/>
-      <c r="J5" s="6"/>
+      <c r="J5" s="6">
+        <v>45940</v>
+      </c>
       <c r="K5" s="6" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>51</v>
+        <v>110</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>19</v>
@@ -7514,13 +7607,13 @@
         <v>36</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="6">
@@ -7534,15 +7627,15 @@
       </c>
       <c r="M6" s="7"/>
     </row>
-    <row r="7" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>19</v>
@@ -7551,33 +7644,35 @@
         <v>36</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I7" s="7"/>
       <c r="J7" s="6">
         <v>45940</v>
       </c>
-      <c r="K7" s="6"/>
+      <c r="K7" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="L7" s="7" t="s">
         <v>22</v>
       </c>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>19</v>
@@ -7586,13 +7681,13 @@
         <v>36</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I8" s="7"/>
       <c r="J8" s="6">
@@ -7606,15 +7701,15 @@
       </c>
       <c r="M8" s="7"/>
     </row>
-    <row r="9" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>19</v>
@@ -7623,13 +7718,13 @@
         <v>36</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="6">
@@ -7643,15 +7738,15 @@
       </c>
       <c r="M9" s="7"/>
     </row>
-    <row r="10" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>19</v>
@@ -7660,13 +7755,13 @@
         <v>36</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I10" s="7"/>
       <c r="J10" s="6">
@@ -7680,15 +7775,15 @@
       </c>
       <c r="M10" s="7"/>
     </row>
-    <row r="11" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>19</v>
@@ -7697,13 +7792,13 @@
         <v>36</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I11" s="7"/>
       <c r="J11" s="6">
@@ -7717,15 +7812,15 @@
       </c>
       <c r="M11" s="7"/>
     </row>
-    <row r="12" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>19</v>
@@ -7734,13 +7829,13 @@
         <v>36</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" s="6">
@@ -7759,10 +7854,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>19</v>
@@ -7771,17 +7866,15 @@
         <v>36</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>79</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="I13" s="7"/>
       <c r="J13" s="6">
         <v>45940</v>
       </c>
@@ -7789,7 +7882,7 @@
         <v>40</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M13" s="7"/>
     </row>
@@ -7798,10 +7891,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>19</v>
@@ -7810,13 +7903,13 @@
         <v>36</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I14" s="7"/>
       <c r="J14" s="6">
@@ -7835,10 +7928,10 @@
         <v>29</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>19</v>
@@ -7847,17 +7940,17 @@
         <v>36</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="6">
-        <v>45940</v>
+        <v>45945</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>40</v>
@@ -7865,17 +7958,19 @@
       <c r="L15" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="M15" s="7"/>
+      <c r="M15" s="9" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="16" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>29</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>19</v>
@@ -7884,13 +7979,13 @@
         <v>36</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I16" s="7"/>
       <c r="J16" s="6">
@@ -7909,23 +8004,19 @@
         <v>30</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
       <c r="G17" s="7"/>
       <c r="H17" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="I17" s="7"/>
       <c r="J17" s="6">
@@ -7939,30 +8030,46 @@
       </c>
       <c r="M17" s="7"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
+    <row r="18" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>19</v>
+      </c>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
+      <c r="H18" s="7" t="s">
+        <v>106</v>
+      </c>
       <c r="I18" s="7"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="7"/>
+      <c r="J18" s="6">
+        <v>45940</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="M18" s="7"/>
     </row>
-    <row r="19" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="135" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>32</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>19</v>
@@ -7971,17 +8078,17 @@
         <v>36</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I19" s="7"/>
       <c r="J19" s="6">
-        <v>45940</v>
+        <v>45945</v>
       </c>
       <c r="K19" s="6" t="s">
         <v>40</v>
@@ -7991,15 +8098,15 @@
       </c>
       <c r="M19" s="7"/>
     </row>
-    <row r="20" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>19</v>
@@ -8008,17 +8115,17 @@
         <v>36</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="I20" s="7"/>
       <c r="J20" s="6">
-        <v>45940</v>
+        <v>45945</v>
       </c>
       <c r="K20" s="6" t="s">
         <v>40</v>
@@ -8028,49 +8135,115 @@
       </c>
       <c r="M20" s="7"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
+    <row r="21" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>97</v>
+      </c>
       <c r="I21" s="7"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="7"/>
+      <c r="J21" s="6">
+        <v>45945</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="M21" s="7"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
+    <row r="22" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>115</v>
+      </c>
       <c r="I22" s="7"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="7"/>
+      <c r="J22" s="6">
+        <v>45945</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="M22" s="7"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
+    <row r="23" spans="1:13" ht="195" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>119</v>
+      </c>
       <c r="I23" s="7"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="7"/>
+      <c r="J23" s="6">
+        <v>45945</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="M23" s="7"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -9831,13 +10004,13 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="L3:L140">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"PENDING"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"PASS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9849,9 +10022,12 @@
       <formula1>INDIRECT("Modulos[MODULOS]")</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="M15" r:id="rId1" xr:uid="{E03BA14B-EB46-4555-B0FE-E6A8B84EE875}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10031,21 +10207,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E158E2AB9B4F924688B558FA982B40CF" ma:contentTypeVersion="3" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ce5f689dcf51305603cb0d070870d6dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="def3e2b2-904e-4359-b966-59b7b32cd06e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="252587ffdfea7067e66d630466c44dd6" ns2:_="">
     <xsd:import namespace="def3e2b2-904e-4359-b966-59b7b32cd06e"/>
@@ -10183,24 +10344,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A2950B-6D37-4A45-BCA2-DEBA33559D5B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CABA5C2-04D8-4DC5-BBFB-FF9AC004B268}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1F0EA96-F162-49AF-B0BE-A54883795866}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10216,4 +10375,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CABA5C2-04D8-4DC5-BBFB-FF9AC004B268}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A2950B-6D37-4A45-BCA2-DEBA33559D5B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modificaciones de testPlant de Fabrizio
</commit_message>
<xml_diff>
--- a/Modelo Test Plan.xlsx
+++ b/Modelo Test Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eva Laura\Documents\PROYECTO DE SISTEMAS III\proyecto\CoderBits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F832D88E-EF25-4644-8279-884CE5A49B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7253DF-0869-4CCD-AC3D-F2E9531BABE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{96765352-7388-4C61-94B8-5077301D3254}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1765" uniqueCount="873">
   <si>
     <t>MODULOS</t>
   </si>
@@ -2752,6 +2752,357 @@
   </si>
   <si>
     <t>Exportacion y descarga de datos si está disponible descargar.</t>
+  </si>
+  <si>
+    <t>https://github.com/alejav0240/CoderBits/issues/41</t>
+  </si>
+  <si>
+    <t>https://github.com/alejav0240/CoderBits/issues/42</t>
+  </si>
+  <si>
+    <t>Visualización de módulos</t>
+  </si>
+  <si>
+    <t>Validar que el panel principal muestre todos los módulos correctamente.</t>
+  </si>
+  <si>
+    <t>1. Acceder al panel principal.2. Verificar que los módulos estén visibles.</t>
+  </si>
+  <si>
+    <t>Acceso con usuario válido.</t>
+  </si>
+  <si>
+    <t>El sistema muestra todos los módulos disponibles.</t>
+  </si>
+  <si>
+    <t>FABRIZIO PAVEL ROLLANO LUNA</t>
+  </si>
+  <si>
+    <t>Navegación entre módulos</t>
+  </si>
+  <si>
+    <t>Validar la correcta navegación entre diferentes módulos del sistema.</t>
+  </si>
+  <si>
+    <t>1. Seleccionar módulo del menú lateral.2. Verificar cambio de vista.</t>
+  </si>
+  <si>
+    <t>Usuario autenticado.</t>
+  </si>
+  <si>
+    <t>El sistema navega correctamente entre módulos.</t>
+  </si>
+  <si>
+    <t>Adaptación responsive</t>
+  </si>
+  <si>
+    <t>Verificar que la interfaz del panel se adapte correctamente a distintas resoluciones de pantalla.</t>
+  </si>
+  <si>
+    <t>1. Acceder al dashboard desde distintos dispositivos.2. Verificar que la interfaz se adapte correctamente.</t>
+  </si>
+  <si>
+    <t>Dispositivos con diferentes resoluciones.</t>
+  </si>
+  <si>
+    <t>La interfaz se adapta correctamente sin pérdida de información.</t>
+  </si>
+  <si>
+    <t>Conexiones</t>
+  </si>
+  <si>
+    <t>Registro de conexiones</t>
+  </si>
+  <si>
+    <t>Validar que las conexiones se registren correctamente y se muestren en la lista.</t>
+  </si>
+  <si>
+    <t>1. Acceder a “Dashboard &gt; Conexions”.2. Registrar una nueva conexión.3. Verificar su aparición en la lista.</t>
+  </si>
+  <si>
+    <t>Datos simulados de conexión.</t>
+  </si>
+  <si>
+    <t>La conexión se guarda correctamente y aparece listada.</t>
+  </si>
+  <si>
+    <t>Búsqueda de conexiones</t>
+  </si>
+  <si>
+    <t>Verificar que la función de búsqueda devuelva resultados coincidentes.</t>
+  </si>
+  <si>
+    <t>Deben existir registros previos.</t>
+  </si>
+  <si>
+    <t>1. Ingresar término en el buscador.2. Ejecutar búsqueda.</t>
+  </si>
+  <si>
+    <t>Texto parcial o completo de la conexión.</t>
+  </si>
+  <si>
+    <t>El sistema muestra solo las coincidencias.</t>
+  </si>
+  <si>
+    <t>Filtro por fecha</t>
+  </si>
+  <si>
+    <t>Validar que los filtros por fecha funcionen correctamente.</t>
+  </si>
+  <si>
+    <t>Deben existir conexiones registradas.</t>
+  </si>
+  <si>
+    <t>1. Aplicar filtro “Today” o “Past 7 days”.2. Verificar resultados filtrados.</t>
+  </si>
+  <si>
+    <t>Conexiones con fechas distintas.</t>
+  </si>
+  <si>
+    <t>Solo se muestran las conexiones en el rango seleccionado.</t>
+  </si>
+  <si>
+    <t>Paginación de registros</t>
+  </si>
+  <si>
+    <t>Validar que los datos de conexión puedan eliminarse correctamente desde la lista.</t>
+  </si>
+  <si>
+    <t>1. Registrar más de 20 conexiones.2. Navegar entre páginas.</t>
+  </si>
+  <si>
+    <t>Registros de conexión simulados.</t>
+  </si>
+  <si>
+    <t>La paginación funciona sin errores.</t>
+  </si>
+  <si>
+    <t>Registro de ataques</t>
+  </si>
+  <si>
+    <t>Confirmar que se puedan editar registros de conexión sin errores.</t>
+  </si>
+  <si>
+    <t>1. Ingresar a “Ataques &gt; Add”.2. Completar campos requeridos.3. Guardar.</t>
+  </si>
+  <si>
+    <t>Datos de ataque simulados.</t>
+  </si>
+  <si>
+    <t>El registro se crea exitosamente.</t>
+  </si>
+  <si>
+    <t>Edición de ataques</t>
+  </si>
+  <si>
+    <t>Verificar que se muestren correctamente los detalles al abrir un registro.</t>
+  </si>
+  <si>
+    <t>Funcionalidad</t>
+  </si>
+  <si>
+    <t>Debe existir un ataque registrado.</t>
+  </si>
+  <si>
+    <t>1. Seleccionar un registro.2. Modificar campos.3. Guardar cambios.</t>
+  </si>
+  <si>
+    <t>Datos actualizados de ataque.</t>
+  </si>
+  <si>
+    <t>El ataque se actualiza correctamente.</t>
+  </si>
+  <si>
+    <t>Eliminación de ataques</t>
+  </si>
+  <si>
+    <t>Validar que los ataques puedan registrarse exitosamente.</t>
+  </si>
+  <si>
+    <t>1. Seleccionar un ataque.2. Eliminar registro.3. Confirmar acción.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>El ataque se elimina correctamente sin afectar otros datos.</t>
+  </si>
+  <si>
+    <t>Registro de mitigaciones</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema muestre todos los ataques registrados en la lista.</t>
+  </si>
+  <si>
+    <t>1. Ingresar a “Mitigaciones &gt; Add”.2. Completar los campos.3. Guardar registro.</t>
+  </si>
+  <si>
+    <t>Datos de prueba de mitigación.</t>
+  </si>
+  <si>
+    <t>El sistema guarda correctamente la mitigación.</t>
+  </si>
+  <si>
+    <t>Validación campo obligatorio Ataque</t>
+  </si>
+  <si>
+    <t>Confirmar que se puedan eliminar ataques de forma segura y controlada.</t>
+  </si>
+  <si>
+    <t>1. Intentar guardar sin seleccionar “Ataque”.</t>
+  </si>
+  <si>
+    <t>Campos vacíos.</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar error de campo obligatorio.</t>
+  </si>
+  <si>
+    <t>Validación de formato IP</t>
+  </si>
+  <si>
+    <t>Verificar que los filtros por tipo de ataque funcionen correctamente.</t>
+  </si>
+  <si>
+    <t>1. Ingresar una IP incorrecta.2. Guardar.</t>
+  </si>
+  <si>
+    <t>IP inválida.</t>
+  </si>
+  <si>
+    <t>El sistema muestra mensaje de error.</t>
+  </si>
+  <si>
+    <t>Creación de ataque desde icono “+”</t>
+  </si>
+  <si>
+    <t>Validar que los ataques puedan ser editados y guardados correctamente.</t>
+  </si>
+  <si>
+    <t>1. Clic en “+” junto a Ataque.2. Crear nuevo ataque.3. Verificar que se vincule.</t>
+  </si>
+  <si>
+    <t>El nuevo ataque se crea y se asocia a la mitigación.</t>
+  </si>
+  <si>
+    <t>Guardado de resultados extensos</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema muestre un mensaje de éxito al guardar una mitigación.</t>
+  </si>
+  <si>
+    <t>1. Ingresar texto largo en “Detalle”.2. Guardar.</t>
+  </si>
+  <si>
+    <t>Texto con más de 1000 caracteres.</t>
+  </si>
+  <si>
+    <t>El sistema guarda sin errores ni cortes.</t>
+  </si>
+  <si>
+    <t>Personales</t>
+  </si>
+  <si>
+    <t>Validar que las mitigaciones estén correctamente asociadas a un ataque.</t>
+  </si>
+  <si>
+    <t>1. Ingresar datos del personal.2. Guardar.</t>
+  </si>
+  <si>
+    <t>Datos personales simulados.</t>
+  </si>
+  <si>
+    <t>El personal se registra correctamente.</t>
+  </si>
+  <si>
+    <t>Edición del personal</t>
+  </si>
+  <si>
+    <t>Confirmar que se guarden correctamente los datos ingresados en los campos de detalle e IP.</t>
+  </si>
+  <si>
+    <t>Debe existir un registro.</t>
+  </si>
+  <si>
+    <t>1. Seleccionar registro.2. Editar.3. Guardar.</t>
+  </si>
+  <si>
+    <t>Nuevos datos personales.</t>
+  </si>
+  <si>
+    <t>El registro se actualiza correctamente.</t>
+  </si>
+  <si>
+    <t>Roles</t>
+  </si>
+  <si>
+    <t>Creación de roles</t>
+  </si>
+  <si>
+    <t>Verificar que el campo “Ejecutado por” funcione correctamente al seleccionar un usuario.</t>
+  </si>
+  <si>
+    <t>1. Ingresar nuevo rol.2. Asignar permisos.3. Guardar.</t>
+  </si>
+  <si>
+    <t>Datos de rol simulados.</t>
+  </si>
+  <si>
+    <t>El rol se crea correctamente.</t>
+  </si>
+  <si>
+    <t>Verificación de permisos por rol</t>
+  </si>
+  <si>
+    <t>Validar que la casilla “Activo” actualice correctamente el estado de la mitigación.</t>
+  </si>
+  <si>
+    <t>Deben existir roles registrados.</t>
+  </si>
+  <si>
+    <t>1. Asignar usuario a rol limitado.2. Intentar acceder a vistas restringidas.</t>
+  </si>
+  <si>
+    <t>Usuario limitado.</t>
+  </si>
+  <si>
+    <t>El sistema bloquea accesos no permitidos.</t>
+  </si>
+  <si>
+    <t>Usuarios</t>
+  </si>
+  <si>
+    <t>Registro de usuarios</t>
+  </si>
+  <si>
+    <t>Verificar que el campo “Resultado” muestre el texto ingresado tras guardar.</t>
+  </si>
+  <si>
+    <t>1. Ingresar usuario nuevo.2. Guardar.</t>
+  </si>
+  <si>
+    <t>Datos simulados de usuario.</t>
+  </si>
+  <si>
+    <t>El usuario se crea correctamente.</t>
+  </si>
+  <si>
+    <t>Cambio de contraseña</t>
+  </si>
+  <si>
+    <t>Validar que el botón “Save” almacene correctamente la mitigación y retorne a la lista.</t>
+  </si>
+  <si>
+    <t>Debe existir usuario registrado.</t>
+  </si>
+  <si>
+    <t>1. Acceder al perfil.2. Cambiar contraseña.3. Verificar autenticación con nueva clave.</t>
+  </si>
+  <si>
+    <t>Contraseña antigua y nueva.</t>
+  </si>
+  <si>
+    <t>El sistema actualiza la contraseña correctamente.</t>
   </si>
 </sst>
 </file>
@@ -2786,12 +3137,18 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -2807,7 +3164,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2836,12 +3193,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="63">
+  <dxfs count="66">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2871,6 +3231,117 @@
           <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
@@ -2961,87 +3432,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center"/>
@@ -8910,54 +9300,54 @@
     <dataField name="Cuenta de Estado (Dropdown)" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="14">
-    <format dxfId="16">
+    <format dxfId="46">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="45">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="44">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="43">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="40">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="39">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="38">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="34">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -9104,60 +9494,60 @@
     <dataField name="Cuenta de Test Case" fld="1" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="16">
-    <format dxfId="32">
+    <format dxfId="62">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="61">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="60">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="59">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="58">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="54">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="53">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="52">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="51">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="50">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -9257,32 +9647,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BEF40B4A-F25E-458D-960B-8087E596FA2C}" name="Modulos" displayName="Modulos" ref="A1:A33" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BEF40B4A-F25E-458D-960B-8087E596FA2C}" name="Modulos" displayName="Modulos" ref="A1:A33" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A1:A33" xr:uid="{BEF40B4A-F25E-458D-960B-8087E596FA2C}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{A3748FA1-9695-4A2D-A595-64BF200E5D1D}" name="MODULOS" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{A3748FA1-9695-4A2D-A595-64BF200E5D1D}" name="MODULOS" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{580B5FFA-030D-4D17-8F6D-90DDF4342984}" name="TestPlan" displayName="TestPlan" ref="A2:M141" headerRowDxfId="59">
-  <autoFilter ref="A2:M141" xr:uid="{580B5FFA-030D-4D17-8F6D-90DDF4342984}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{580B5FFA-030D-4D17-8F6D-90DDF4342984}" name="TestPlan" displayName="TestPlan" ref="A2:M162" headerRowDxfId="32">
+  <autoFilter ref="A2:M162" xr:uid="{580B5FFA-030D-4D17-8F6D-90DDF4342984}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{7F95280F-E669-4A5D-AEDF-FCAAAC81F275}" name="Modulo (Dropdown)" totalsRowLabel="Total" dataDxfId="58" totalsRowDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{E775B39B-DEB6-4123-A65F-A37EDA4383A3}" name="Test Case" dataDxfId="56" totalsRowDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{4E500E60-0861-4EF2-B610-79885F5EF7FD}" name="Descripción" dataDxfId="54" totalsRowDxfId="53"/>
-    <tableColumn id="14" xr3:uid="{D149BE2F-3E66-4E54-8D0E-BA4D69F73794}" name="Tipo/s de Prueba" dataDxfId="52" totalsRowDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{48166857-FFB0-4E91-A69A-8A057DEBB914}" name="Precondiciones" dataDxfId="50" totalsRowDxfId="49"/>
-    <tableColumn id="13" xr3:uid="{09440620-A437-484D-9292-769D8C979710}" name="Pasos a seguir" dataDxfId="48" totalsRowDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{25FFAFC4-E636-4C78-8EC4-9B105CD6EC6A}" name="Datos de Prueba" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{5C319188-663F-4BD1-ADB0-A93CF2F134F5}" name="Resultado Esperado" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{AC65C1EE-D520-403E-8171-F3B42F898A90}" name="Resultado Actual (Si falla)" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{67BFFC43-BD7A-400D-BCA5-7641851369E7}" name="Ultima ejecución (Fecha)" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="10" xr3:uid="{AF2F4479-94ED-46CC-8F6A-9945904E34B4}" name="Encargado de Prueba" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{1AE568CA-11EA-494D-A158-098CEC0427F1}" name="Estado (Dropdown)" dataDxfId="36" totalsRowDxfId="35"/>
-    <tableColumn id="9" xr3:uid="{D7CC1236-1B17-4FEE-A062-7A6AF5789012}" name="Comentario" totalsRowFunction="count" dataDxfId="34" totalsRowDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{7F95280F-E669-4A5D-AEDF-FCAAAC81F275}" name="Modulo (Dropdown)" totalsRowLabel="Total" dataDxfId="30" totalsRowDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{E775B39B-DEB6-4123-A65F-A37EDA4383A3}" name="Test Case" dataDxfId="28" totalsRowDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{4E500E60-0861-4EF2-B610-79885F5EF7FD}" name="Descripción" dataDxfId="26" totalsRowDxfId="27"/>
+    <tableColumn id="14" xr3:uid="{D149BE2F-3E66-4E54-8D0E-BA4D69F73794}" name="Tipo/s de Prueba" dataDxfId="24" totalsRowDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{48166857-FFB0-4E91-A69A-8A057DEBB914}" name="Precondiciones" dataDxfId="22" totalsRowDxfId="23"/>
+    <tableColumn id="13" xr3:uid="{09440620-A437-484D-9292-769D8C979710}" name="Pasos a seguir" dataDxfId="20" totalsRowDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{25FFAFC4-E636-4C78-8EC4-9B105CD6EC6A}" name="Datos de Prueba" dataDxfId="18" totalsRowDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{5C319188-663F-4BD1-ADB0-A93CF2F134F5}" name="Resultado Esperado" dataDxfId="16" totalsRowDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{AC65C1EE-D520-403E-8171-F3B42F898A90}" name="Resultado Actual (Si falla)" dataDxfId="14" totalsRowDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{67BFFC43-BD7A-400D-BCA5-7641851369E7}" name="Ultima ejecución (Fecha)" dataDxfId="12" totalsRowDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{AF2F4479-94ED-46CC-8F6A-9945904E34B4}" name="Encargado de Prueba" dataDxfId="10" totalsRowDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{1AE568CA-11EA-494D-A158-098CEC0427F1}" name="Estado (Dropdown)" dataDxfId="8" totalsRowDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{D7CC1236-1B17-4FEE-A062-7A6AF5789012}" name="Comentario" totalsRowFunction="count" dataDxfId="6" totalsRowDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9730,7 +10120,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D9AFB2-4BAC-4EFB-A2E7-92EA3A8E1FBC}">
-  <dimension ref="A2:M141"/>
+  <dimension ref="A2:M162"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.85546875" customWidth="1"/>
@@ -14774,7 +15164,9 @@
       <c r="L137" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="M137" s="7"/>
+      <c r="M137" s="9" t="s">
+        <v>756</v>
+      </c>
     </row>
     <row r="138" spans="1:13" ht="45">
       <c r="A138" s="7" t="s">
@@ -14813,7 +15205,9 @@
       <c r="L138" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="M138" s="7"/>
+      <c r="M138" s="9" t="s">
+        <v>757</v>
+      </c>
     </row>
     <row r="139" spans="1:13" ht="60">
       <c r="A139" s="7" t="s">
@@ -14926,9 +15320,797 @@
       </c>
       <c r="M141" s="7"/>
     </row>
+    <row r="142" spans="1:13" ht="45">
+      <c r="A142" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B142" s="7" t="s">
+        <v>758</v>
+      </c>
+      <c r="C142" s="7" t="s">
+        <v>759</v>
+      </c>
+      <c r="D142" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E142" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F142" s="7" t="s">
+        <v>760</v>
+      </c>
+      <c r="G142" s="7" t="s">
+        <v>761</v>
+      </c>
+      <c r="H142" s="7" t="s">
+        <v>762</v>
+      </c>
+      <c r="I142" s="7"/>
+      <c r="J142" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K142" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L142" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M142" s="7"/>
+    </row>
+    <row r="143" spans="1:13" ht="45">
+      <c r="A143" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B143" s="7" t="s">
+        <v>764</v>
+      </c>
+      <c r="C143" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="D143" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E143" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F143" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="G143" s="7" t="s">
+        <v>767</v>
+      </c>
+      <c r="H143" s="7" t="s">
+        <v>768</v>
+      </c>
+      <c r="I143" s="7"/>
+      <c r="J143" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K143" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L143" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M143" s="7"/>
+    </row>
+    <row r="144" spans="1:13" ht="60">
+      <c r="A144" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B144" s="7" t="s">
+        <v>769</v>
+      </c>
+      <c r="C144" s="7" t="s">
+        <v>770</v>
+      </c>
+      <c r="D144" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E144" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F144" s="7" t="s">
+        <v>771</v>
+      </c>
+      <c r="G144" s="7" t="s">
+        <v>772</v>
+      </c>
+      <c r="H144" s="7" t="s">
+        <v>773</v>
+      </c>
+      <c r="I144" s="7"/>
+      <c r="J144" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K144" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L144" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M144" s="7"/>
+    </row>
+    <row r="145" spans="1:13" ht="60">
+      <c r="A145" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="B145" s="7" t="s">
+        <v>775</v>
+      </c>
+      <c r="C145" s="7" t="s">
+        <v>776</v>
+      </c>
+      <c r="D145" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E145" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F145" s="7" t="s">
+        <v>777</v>
+      </c>
+      <c r="G145" s="7" t="s">
+        <v>778</v>
+      </c>
+      <c r="H145" s="7" t="s">
+        <v>779</v>
+      </c>
+      <c r="I145" s="7"/>
+      <c r="J145" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K145" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L145" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M145" s="7"/>
+    </row>
+    <row r="146" spans="1:13" ht="30">
+      <c r="A146" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="B146" s="7" t="s">
+        <v>780</v>
+      </c>
+      <c r="C146" s="7" t="s">
+        <v>781</v>
+      </c>
+      <c r="D146" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E146" s="7" t="s">
+        <v>782</v>
+      </c>
+      <c r="F146" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="G146" s="7" t="s">
+        <v>784</v>
+      </c>
+      <c r="H146" s="7" t="s">
+        <v>785</v>
+      </c>
+      <c r="I146" s="7"/>
+      <c r="J146" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K146" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L146" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M146" s="7"/>
+    </row>
+    <row r="147" spans="1:13" ht="45">
+      <c r="A147" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="B147" s="7" t="s">
+        <v>786</v>
+      </c>
+      <c r="C147" s="7" t="s">
+        <v>787</v>
+      </c>
+      <c r="D147" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E147" s="7" t="s">
+        <v>788</v>
+      </c>
+      <c r="F147" s="7" t="s">
+        <v>789</v>
+      </c>
+      <c r="G147" s="7" t="s">
+        <v>790</v>
+      </c>
+      <c r="H147" s="7" t="s">
+        <v>791</v>
+      </c>
+      <c r="I147" s="7"/>
+      <c r="J147" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K147" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L147" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M147" s="7"/>
+    </row>
+    <row r="148" spans="1:13" ht="45">
+      <c r="A148" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="B148" s="7" t="s">
+        <v>792</v>
+      </c>
+      <c r="C148" s="7" t="s">
+        <v>793</v>
+      </c>
+      <c r="D148" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E148" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F148" s="7" t="s">
+        <v>794</v>
+      </c>
+      <c r="G148" s="7" t="s">
+        <v>795</v>
+      </c>
+      <c r="H148" s="7" t="s">
+        <v>796</v>
+      </c>
+      <c r="I148" s="7"/>
+      <c r="J148" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K148" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L148" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M148" s="7"/>
+    </row>
+    <row r="149" spans="1:13" ht="45">
+      <c r="A149" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>797</v>
+      </c>
+      <c r="C149" s="7" t="s">
+        <v>798</v>
+      </c>
+      <c r="D149" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E149" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F149" s="7" t="s">
+        <v>799</v>
+      </c>
+      <c r="G149" s="7" t="s">
+        <v>800</v>
+      </c>
+      <c r="H149" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="I149" s="7"/>
+      <c r="J149" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K149" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L149" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M149" s="7"/>
+    </row>
+    <row r="150" spans="1:13" ht="45">
+      <c r="A150" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B150" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="C150" s="7" t="s">
+        <v>803</v>
+      </c>
+      <c r="D150" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="E150" s="7" t="s">
+        <v>805</v>
+      </c>
+      <c r="F150" s="7" t="s">
+        <v>806</v>
+      </c>
+      <c r="G150" s="7" t="s">
+        <v>807</v>
+      </c>
+      <c r="H150" s="7" t="s">
+        <v>808</v>
+      </c>
+      <c r="I150" s="7"/>
+      <c r="J150" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K150" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L150" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M150" s="7"/>
+    </row>
+    <row r="151" spans="1:13" ht="45">
+      <c r="A151" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B151" s="7" t="s">
+        <v>809</v>
+      </c>
+      <c r="C151" s="7" t="s">
+        <v>810</v>
+      </c>
+      <c r="D151" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="E151" s="7" t="s">
+        <v>805</v>
+      </c>
+      <c r="F151" s="7" t="s">
+        <v>811</v>
+      </c>
+      <c r="G151" s="7" t="s">
+        <v>812</v>
+      </c>
+      <c r="H151" s="7" t="s">
+        <v>813</v>
+      </c>
+      <c r="I151" s="7"/>
+      <c r="J151" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K151" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L151" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M151" s="7"/>
+    </row>
+    <row r="152" spans="1:13" ht="45">
+      <c r="A152" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B152" s="7" t="s">
+        <v>814</v>
+      </c>
+      <c r="C152" s="7" t="s">
+        <v>815</v>
+      </c>
+      <c r="D152" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E152" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F152" s="7" t="s">
+        <v>816</v>
+      </c>
+      <c r="G152" s="7" t="s">
+        <v>817</v>
+      </c>
+      <c r="H152" s="7" t="s">
+        <v>818</v>
+      </c>
+      <c r="I152" s="7"/>
+      <c r="J152" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K152" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L152" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M152" s="7"/>
+    </row>
+    <row r="153" spans="1:13" ht="30">
+      <c r="A153" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>819</v>
+      </c>
+      <c r="C153" s="7" t="s">
+        <v>820</v>
+      </c>
+      <c r="D153" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E153" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F153" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="G153" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="H153" s="7" t="s">
+        <v>823</v>
+      </c>
+      <c r="I153" s="7"/>
+      <c r="J153" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K153" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L153" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M153" s="7"/>
+    </row>
+    <row r="154" spans="1:13" ht="30">
+      <c r="A154" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B154" s="7" t="s">
+        <v>824</v>
+      </c>
+      <c r="C154" s="7" t="s">
+        <v>825</v>
+      </c>
+      <c r="D154" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E154" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F154" s="7" t="s">
+        <v>826</v>
+      </c>
+      <c r="G154" s="7" t="s">
+        <v>827</v>
+      </c>
+      <c r="H154" s="7" t="s">
+        <v>828</v>
+      </c>
+      <c r="I154" s="7"/>
+      <c r="J154" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K154" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L154" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M154" s="7"/>
+    </row>
+    <row r="155" spans="1:13" ht="45">
+      <c r="A155" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>829</v>
+      </c>
+      <c r="C155" s="7" t="s">
+        <v>830</v>
+      </c>
+      <c r="D155" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="E155" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F155" s="7" t="s">
+        <v>831</v>
+      </c>
+      <c r="G155" s="7" t="s">
+        <v>800</v>
+      </c>
+      <c r="H155" s="7" t="s">
+        <v>832</v>
+      </c>
+      <c r="I155" s="7"/>
+      <c r="J155" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K155" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L155" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M155" s="7"/>
+    </row>
+    <row r="156" spans="1:13" ht="45">
+      <c r="A156" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B156" s="7" t="s">
+        <v>833</v>
+      </c>
+      <c r="C156" s="7" t="s">
+        <v>834</v>
+      </c>
+      <c r="D156" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="E156" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F156" s="7" t="s">
+        <v>835</v>
+      </c>
+      <c r="G156" s="7" t="s">
+        <v>836</v>
+      </c>
+      <c r="H156" s="7" t="s">
+        <v>837</v>
+      </c>
+      <c r="I156" s="7"/>
+      <c r="J156" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K156" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L156" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M156" s="7"/>
+    </row>
+    <row r="157" spans="1:13" ht="30">
+      <c r="A157" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C157" s="7" t="s">
+        <v>839</v>
+      </c>
+      <c r="D157" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E157" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F157" s="7" t="s">
+        <v>840</v>
+      </c>
+      <c r="G157" s="7" t="s">
+        <v>841</v>
+      </c>
+      <c r="H157" s="7" t="s">
+        <v>842</v>
+      </c>
+      <c r="I157" s="7"/>
+      <c r="J157" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K157" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L157" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M157" s="7"/>
+    </row>
+    <row r="158" spans="1:13" ht="45">
+      <c r="A158" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="B158" s="7" t="s">
+        <v>843</v>
+      </c>
+      <c r="C158" s="7" t="s">
+        <v>844</v>
+      </c>
+      <c r="D158" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="E158" s="7" t="s">
+        <v>845</v>
+      </c>
+      <c r="F158" s="7" t="s">
+        <v>846</v>
+      </c>
+      <c r="G158" s="7" t="s">
+        <v>847</v>
+      </c>
+      <c r="H158" s="7" t="s">
+        <v>848</v>
+      </c>
+      <c r="I158" s="7"/>
+      <c r="J158" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K158" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L158" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M158" s="7"/>
+    </row>
+    <row r="159" spans="1:13" ht="45">
+      <c r="A159" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>850</v>
+      </c>
+      <c r="C159" s="7" t="s">
+        <v>851</v>
+      </c>
+      <c r="D159" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E159" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F159" s="7" t="s">
+        <v>852</v>
+      </c>
+      <c r="G159" s="7" t="s">
+        <v>853</v>
+      </c>
+      <c r="H159" s="7" t="s">
+        <v>854</v>
+      </c>
+      <c r="I159" s="7"/>
+      <c r="J159" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K159" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L159" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M159" s="7"/>
+    </row>
+    <row r="160" spans="1:13" ht="45">
+      <c r="A160" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="B160" s="7" t="s">
+        <v>855</v>
+      </c>
+      <c r="C160" s="7" t="s">
+        <v>856</v>
+      </c>
+      <c r="D160" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E160" s="7" t="s">
+        <v>857</v>
+      </c>
+      <c r="F160" s="7" t="s">
+        <v>858</v>
+      </c>
+      <c r="G160" s="7" t="s">
+        <v>859</v>
+      </c>
+      <c r="H160" s="7" t="s">
+        <v>860</v>
+      </c>
+      <c r="I160" s="7"/>
+      <c r="J160" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K160" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L160" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M160" s="7"/>
+    </row>
+    <row r="161" spans="1:13" ht="30">
+      <c r="A161" s="7" t="s">
+        <v>861</v>
+      </c>
+      <c r="B161" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="C161" s="7" t="s">
+        <v>863</v>
+      </c>
+      <c r="D161" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E161" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F161" s="7" t="s">
+        <v>864</v>
+      </c>
+      <c r="G161" s="7" t="s">
+        <v>865</v>
+      </c>
+      <c r="H161" s="7" t="s">
+        <v>866</v>
+      </c>
+      <c r="I161" s="7"/>
+      <c r="J161" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K161" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L161" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M161" s="7"/>
+    </row>
+    <row r="162" spans="1:13" ht="45">
+      <c r="A162" s="7" t="s">
+        <v>861</v>
+      </c>
+      <c r="B162" s="7" t="s">
+        <v>867</v>
+      </c>
+      <c r="C162" s="7" t="s">
+        <v>868</v>
+      </c>
+      <c r="D162" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E162" s="7" t="s">
+        <v>869</v>
+      </c>
+      <c r="F162" s="7" t="s">
+        <v>870</v>
+      </c>
+      <c r="G162" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="H162" s="7" t="s">
+        <v>872</v>
+      </c>
+      <c r="I162" s="7"/>
+      <c r="J162" s="6">
+        <v>45950</v>
+      </c>
+      <c r="K162" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="L162" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M162" s="7"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="L3:L134 L135:M135 L136:L140">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>"PENDING"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"PASS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
+      <formula>"FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L142:L162">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"PENDING"</formula>
     </cfRule>
@@ -14940,19 +16122,21 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A141" xr:uid="{F4675041-A1B8-4B65-822E-23AD6AB864A0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A162" xr:uid="{F4675041-A1B8-4B65-822E-23AD6AB864A0}">
       <formula1>INDIRECT("Modulos[MODULOS]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M135 L3:L141" xr:uid="{1E8D2D6D-4EE7-40E2-A622-3458BDCF08AD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M135 L3:L162" xr:uid="{1E8D2D6D-4EE7-40E2-A622-3458BDCF08AD}">
       <formula1>"PASS,PENDING,FAIL"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="M15" r:id="rId1" xr:uid="{E03BA14B-EB46-4555-B0FE-E6A8B84EE875}"/>
+    <hyperlink ref="M137" r:id="rId2" xr:uid="{76C22D69-B896-4F17-9D14-9568E036A5E6}"/>
+    <hyperlink ref="M138" r:id="rId3" xr:uid="{B3EE788D-8E23-4A38-9959-7347F6F58207}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -15132,9 +16316,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -15276,19 +16463,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CABA5C2-04D8-4DC5-BBFB-FF9AC004B268}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A2950B-6D37-4A45-BCA2-DEBA33559D5B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -15312,9 +16495,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A2950B-6D37-4A45-BCA2-DEBA33559D5B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CABA5C2-04D8-4DC5-BBFB-FF9AC004B268}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Se implemento el modelo
</commit_message>
<xml_diff>
--- a/Modelo Test Plan.xlsx
+++ b/Modelo Test Plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alumno\CoderBits\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiro\CoderBits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD6634C-5DF2-4E15-B1DF-93BE23FD02D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF9F9C59-B031-4841-905A-833D149FEAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{96765352-7388-4C61-94B8-5077301D3254}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{96765352-7388-4C61-94B8-5077301D3254}"/>
   </bookViews>
   <sheets>
     <sheet name="Gestion de Modulos" sheetId="4" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1742" uniqueCount="865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1760" uniqueCount="876">
   <si>
     <t>MODULOS</t>
   </si>
@@ -3047,12 +3047,45 @@
   <si>
     <t>Validacion de que el numero de telefono solo tenga valores numericos</t>
   </si>
+  <si>
+    <t>Bloqueo a nivel firewall</t>
+  </si>
+  <si>
+    <t>Desbloqueo a nivel firewall</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema tiene que bloquear a nivel firewall la ip atacante</t>
+  </si>
+  <si>
+    <t>Verificar que el sistema tiene que desbloquear a nivel firewall la ip atacante</t>
+  </si>
+  <si>
+    <t>Unitaria</t>
+  </si>
+  <si>
+    <t>Mitigaciones registradas disponibles</t>
+  </si>
+  <si>
+    <t>Mitigaciones bloqueadas</t>
+  </si>
+  <si>
+    <t>1. Iniciar sesion 2. Iniciar el monitoreo de red 3. realizar ataque de prueba 4. Mitigar manual mente</t>
+  </si>
+  <si>
+    <t>1. Iniciar sesion 2. Iniciar el monitoreo de red 3. Desbloquear ip bloqueada</t>
+  </si>
+  <si>
+    <t>Se bloquea la ip del atacante</t>
+  </si>
+  <si>
+    <t>Se desbloquea la ip del atacante</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3070,6 +3103,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3108,7 +3149,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3143,12 +3184,74 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="51">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3298,65 +3401,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center"/>
@@ -4648,6 +4692,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4655,7 +4700,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:gradFill flip="none" rotWithShape="1">
@@ -5199,6 +5243,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5206,7 +5251,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:gradFill flip="none" rotWithShape="1">
@@ -9231,54 +9275,54 @@
     <dataField name="Cuenta de Estado (Dropdown)" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="14">
-    <format dxfId="19">
+    <format dxfId="31">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="30">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="29">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="25">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="24">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="23">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="19">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -9425,60 +9469,60 @@
     <dataField name="Cuenta de Test Case" fld="1" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="16">
-    <format dxfId="35">
+    <format dxfId="47">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="34">
+    <format dxfId="46">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="45">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="44">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="43">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="39">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="38">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="37">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="36">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="35">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -9588,21 +9632,21 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{343BA946-EF1B-4A3B-B511-74A6334C62D3}" name="Tabla1" displayName="Tabla1" ref="A1:L160" totalsRowShown="0">
-  <autoFilter ref="A1:L160" xr:uid="{343BA946-EF1B-4A3B-B511-74A6334C62D3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{343BA946-EF1B-4A3B-B511-74A6334C62D3}" name="Tabla1" displayName="Tabla1" ref="A1:L162" totalsRowShown="0">
+  <autoFilter ref="A1:L162" xr:uid="{343BA946-EF1B-4A3B-B511-74A6334C62D3}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9B76ED1C-581E-403B-9039-C4D1437837BF}" name="Columna1" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{B227DD10-4412-4DA1-B9AE-57DBBAAC5FDB}" name="Columna2" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{946681D4-26C8-4625-A0B6-192416560D49}" name="Descripción" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{1B53AA13-C73C-4BDB-96DD-F68A91E0C473}" name="Tipo/s de Prueba" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{38F51641-8D65-4D91-9238-C57B7E0DC8C4}" name="Precondiciones" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{F67DADA5-19EF-41E4-9B0E-3EB1E6E4AEC7}" name="Pasos a seguir" dataDxfId="42"/>
-    <tableColumn id="7" xr3:uid="{1E37B7C6-6237-424F-9825-DBAC920A3A92}" name="Datos de Prueba" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{6808706D-288F-4E5F-B1EE-9FC3C5DA1057}" name="Resultado Esperado" dataDxfId="40"/>
-    <tableColumn id="9" xr3:uid="{2D9093F3-889A-450D-9A36-E88B55FE392C}" name="Resultado Actual (Si falla)" dataDxfId="39"/>
-    <tableColumn id="10" xr3:uid="{1DD114CA-C7C7-4EE6-9D13-890DFE1B49F9}" name="Ultima ejecución (Fecha)" dataDxfId="38"/>
-    <tableColumn id="11" xr3:uid="{78CB6362-EDEC-4F76-AA97-664327DEED9B}" name="Encargado de Prueba" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{E14C667D-B48D-4C28-B1C7-EA7F85B8361A}" name="Estado (Dropdown)" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{9B76ED1C-581E-403B-9039-C4D1437837BF}" name="Columna1" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{B227DD10-4412-4DA1-B9AE-57DBBAAC5FDB}" name="Columna2" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{946681D4-26C8-4625-A0B6-192416560D49}" name="Descripción" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{1B53AA13-C73C-4BDB-96DD-F68A91E0C473}" name="Tipo/s de Prueba" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{38F51641-8D65-4D91-9238-C57B7E0DC8C4}" name="Precondiciones" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{F67DADA5-19EF-41E4-9B0E-3EB1E6E4AEC7}" name="Pasos a seguir" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{1E37B7C6-6237-424F-9825-DBAC920A3A92}" name="Datos de Prueba" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{6808706D-288F-4E5F-B1EE-9FC3C5DA1057}" name="Resultado Esperado" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{2D9093F3-889A-450D-9A36-E88B55FE392C}" name="Resultado Actual (Si falla)" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{1DD114CA-C7C7-4EE6-9D13-890DFE1B49F9}" name="Ultima ejecución (Fecha)" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{78CB6362-EDEC-4F76-AA97-664327DEED9B}" name="Encargado de Prueba" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{E14C667D-B48D-4C28-B1C7-EA7F85B8361A}" name="Estado (Dropdown)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9926,120 +9970,120 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ACCE336-D829-4280-938B-27FEC42D7852}">
   <dimension ref="A1:A33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="24.75" customHeight="1">
+    <row r="2" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="24.75" customHeight="1">
+    <row r="3" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="24.75" customHeight="1">
+    <row r="4" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="24.75" customHeight="1">
+    <row r="5" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="24.75" customHeight="1">
+    <row r="6" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="24.75" customHeight="1">
+    <row r="7" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="24.75" customHeight="1">
+    <row r="8" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="24.75" customHeight="1">
+    <row r="9" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="24.75" customHeight="1">
+    <row r="10" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="24.75" customHeight="1">
+    <row r="11" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="24.75" customHeight="1">
+    <row r="12" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="24.75" customHeight="1">
+    <row r="13" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="24.75" customHeight="1">
+    <row r="14" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="24.75" customHeight="1">
+    <row r="15" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="24.75" customHeight="1">
+    <row r="16" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="24.75" customHeight="1">
+    <row r="17" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="24.75" customHeight="1">
+    <row r="18" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="24.75" customHeight="1">
+    <row r="19" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="21" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="22" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="23" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="24" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="25" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="26" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="27" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="28" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="29" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="30" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="31" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="32" spans="1:1" ht="24.75" customHeight="1"/>
-    <row r="33" ht="24.75" customHeight="1"/>
+    <row r="20" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -10051,23 +10095,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D9AFB2-4BAC-4EFB-A2E7-92EA3A8E1FBC}">
   <dimension ref="A1:N184"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.875" customWidth="1"/>
-    <col min="2" max="2" width="30.875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="37.375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="37.375" customWidth="1"/>
-    <col min="5" max="5" width="31.75" style="2" customWidth="1"/>
-    <col min="6" max="6" width="49.875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="39.375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="33.875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="31.375" customWidth="1"/>
-    <col min="10" max="11" width="30.375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16.375" customWidth="1"/>
-    <col min="13" max="13" width="36.125" customWidth="1"/>
+    <col min="1" max="1" width="22.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37.42578125" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="49.85546875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="39.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="33.85546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="31.42578125" customWidth="1"/>
+    <col min="10" max="11" width="30.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16.42578125" customWidth="1"/>
+    <col min="13" max="13" width="36.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.5">
+    <row r="1" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -10105,7 +10149,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="2" customFormat="1">
+    <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2"/>
       <c r="D2"/>
       <c r="I2"/>
@@ -10119,7 +10163,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="41.25" customHeight="1">
+    <row r="3" spans="1:14" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
@@ -10159,7 +10203,7 @@
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
     </row>
-    <row r="4" spans="1:14" ht="114">
+    <row r="4" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
@@ -10197,7 +10241,7 @@
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
     </row>
-    <row r="5" spans="1:14" ht="114">
+    <row r="5" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
@@ -10235,7 +10279,7 @@
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
     </row>
-    <row r="6" spans="1:14" ht="114">
+    <row r="6" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
@@ -10273,7 +10317,7 @@
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
     </row>
-    <row r="7" spans="1:14" ht="114">
+    <row r="7" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>2</v>
       </c>
@@ -10311,7 +10355,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
     </row>
-    <row r="8" spans="1:14" ht="114">
+    <row r="8" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>2</v>
       </c>
@@ -10349,7 +10393,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
     </row>
-    <row r="9" spans="1:14" ht="114">
+    <row r="9" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>2</v>
       </c>
@@ -10387,7 +10431,7 @@
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
     </row>
-    <row r="10" spans="1:14" ht="114">
+    <row r="10" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>2</v>
       </c>
@@ -10425,7 +10469,7 @@
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
     </row>
-    <row r="11" spans="1:14" ht="114">
+    <row r="11" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>2</v>
       </c>
@@ -10463,7 +10507,7 @@
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>
     </row>
-    <row r="12" spans="1:14" ht="42.75">
+    <row r="12" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>3</v>
       </c>
@@ -10501,7 +10545,7 @@
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
     </row>
-    <row r="13" spans="1:14" ht="42.75">
+    <row r="13" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>3</v>
       </c>
@@ -10541,7 +10585,7 @@
       </c>
       <c r="N13" s="7"/>
     </row>
-    <row r="14" spans="1:14" ht="28.5">
+    <row r="14" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>4</v>
       </c>
@@ -10579,7 +10623,7 @@
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
     </row>
-    <row r="15" spans="1:14" ht="28.5">
+    <row r="15" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>4</v>
       </c>
@@ -10617,7 +10661,7 @@
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
     </row>
-    <row r="16" spans="1:14" ht="42.75">
+    <row r="16" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>5</v>
       </c>
@@ -10653,7 +10697,7 @@
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
     </row>
-    <row r="17" spans="1:14" ht="42.75">
+    <row r="17" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>5</v>
       </c>
@@ -10689,7 +10733,7 @@
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
     </row>
-    <row r="18" spans="1:14" ht="128.25">
+    <row r="18" spans="1:14" ht="135" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>7</v>
       </c>
@@ -10727,7 +10771,7 @@
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
     </row>
-    <row r="19" spans="1:14" ht="42.75">
+    <row r="19" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>7</v>
       </c>
@@ -10765,7 +10809,7 @@
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
     </row>
-    <row r="20" spans="1:14" ht="42.75">
+    <row r="20" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
@@ -10803,7 +10847,7 @@
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
     </row>
-    <row r="21" spans="1:14" ht="71.25">
+    <row r="21" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>9</v>
       </c>
@@ -10841,7 +10885,7 @@
       <c r="M21" s="7"/>
       <c r="N21" s="7"/>
     </row>
-    <row r="22" spans="1:14" ht="185.25">
+    <row r="22" spans="1:14" ht="195" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>9</v>
       </c>
@@ -10881,7 +10925,7 @@
       </c>
       <c r="N22" s="7"/>
     </row>
-    <row r="23" spans="1:14" ht="128.25">
+    <row r="23" spans="1:14" ht="135" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>5</v>
       </c>
@@ -10920,7 +10964,7 @@
       </c>
       <c r="N23" s="7"/>
     </row>
-    <row r="24" spans="1:14" ht="28.5">
+    <row r="24" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>10</v>
       </c>
@@ -10957,7 +11001,7 @@
       </c>
       <c r="N24" s="7"/>
     </row>
-    <row r="25" spans="1:14" ht="42.75">
+    <row r="25" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>10</v>
       </c>
@@ -10994,7 +11038,7 @@
       </c>
       <c r="N25" s="7"/>
     </row>
-    <row r="26" spans="1:14" ht="42.75">
+    <row r="26" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>10</v>
       </c>
@@ -11031,7 +11075,7 @@
       </c>
       <c r="N26" s="7"/>
     </row>
-    <row r="27" spans="1:14" ht="42.75">
+    <row r="27" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>10</v>
       </c>
@@ -11068,7 +11112,7 @@
       </c>
       <c r="N27" s="7"/>
     </row>
-    <row r="28" spans="1:14" ht="28.5">
+    <row r="28" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>10</v>
       </c>
@@ -11105,7 +11149,7 @@
       </c>
       <c r="N28" s="7"/>
     </row>
-    <row r="29" spans="1:14" ht="42.75">
+    <row r="29" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>10</v>
       </c>
@@ -11142,7 +11186,7 @@
       </c>
       <c r="N29" s="7"/>
     </row>
-    <row r="30" spans="1:14" ht="28.5">
+    <row r="30" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>10</v>
       </c>
@@ -11179,7 +11223,7 @@
       </c>
       <c r="N30" s="7"/>
     </row>
-    <row r="31" spans="1:14" ht="28.5">
+    <row r="31" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>10</v>
       </c>
@@ -11216,7 +11260,7 @@
       </c>
       <c r="N31" s="7"/>
     </row>
-    <row r="32" spans="1:14" ht="28.5">
+    <row r="32" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>10</v>
       </c>
@@ -11253,7 +11297,7 @@
       </c>
       <c r="N32" s="7"/>
     </row>
-    <row r="33" spans="1:14" ht="28.5">
+    <row r="33" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>10</v>
       </c>
@@ -11291,7 +11335,7 @@
       <c r="M33" s="7"/>
       <c r="N33" s="7"/>
     </row>
-    <row r="34" spans="1:14" ht="42.75">
+    <row r="34" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>1</v>
       </c>
@@ -11329,7 +11373,7 @@
       <c r="M34" s="7"/>
       <c r="N34" s="7"/>
     </row>
-    <row r="35" spans="1:14" ht="57">
+    <row r="35" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>1</v>
       </c>
@@ -11367,7 +11411,7 @@
       <c r="M35" s="7"/>
       <c r="N35" s="7"/>
     </row>
-    <row r="36" spans="1:14" ht="57">
+    <row r="36" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>1</v>
       </c>
@@ -11405,7 +11449,7 @@
       <c r="M36" s="7"/>
       <c r="N36" s="7"/>
     </row>
-    <row r="37" spans="1:14" ht="42.75">
+    <row r="37" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>1</v>
       </c>
@@ -11443,7 +11487,7 @@
       <c r="M37" s="7"/>
       <c r="N37" s="7"/>
     </row>
-    <row r="38" spans="1:14" ht="42.75">
+    <row r="38" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>1</v>
       </c>
@@ -11481,7 +11525,7 @@
       <c r="M38" s="7"/>
       <c r="N38" s="7"/>
     </row>
-    <row r="39" spans="1:14" ht="42.75">
+    <row r="39" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>1</v>
       </c>
@@ -11519,7 +11563,7 @@
       <c r="M39" s="7"/>
       <c r="N39" s="7"/>
     </row>
-    <row r="40" spans="1:14" ht="42.75">
+    <row r="40" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>1</v>
       </c>
@@ -11557,7 +11601,7 @@
       <c r="M40" s="7"/>
       <c r="N40" s="7"/>
     </row>
-    <row r="41" spans="1:14" ht="42.75">
+    <row r="41" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>1</v>
       </c>
@@ -11595,7 +11639,7 @@
       <c r="M41" s="7"/>
       <c r="N41" s="7"/>
     </row>
-    <row r="42" spans="1:14" ht="42.75">
+    <row r="42" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>1</v>
       </c>
@@ -11633,7 +11677,7 @@
       <c r="M42" s="7"/>
       <c r="N42" s="7"/>
     </row>
-    <row r="43" spans="1:14" ht="57">
+    <row r="43" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>1</v>
       </c>
@@ -11671,7 +11715,7 @@
       <c r="M43" s="7"/>
       <c r="N43" s="7"/>
     </row>
-    <row r="44" spans="1:14" ht="42.75">
+    <row r="44" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>1</v>
       </c>
@@ -11709,7 +11753,7 @@
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
     </row>
-    <row r="45" spans="1:14" ht="42.75">
+    <row r="45" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>1</v>
       </c>
@@ -11747,7 +11791,7 @@
       <c r="M45" s="7"/>
       <c r="N45" s="7"/>
     </row>
-    <row r="46" spans="1:14" ht="57">
+    <row r="46" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>1</v>
       </c>
@@ -11785,7 +11829,7 @@
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
     </row>
-    <row r="47" spans="1:14" ht="57">
+    <row r="47" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>1</v>
       </c>
@@ -11823,7 +11867,7 @@
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
     </row>
-    <row r="48" spans="1:14" ht="42.75">
+    <row r="48" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>1</v>
       </c>
@@ -11861,7 +11905,7 @@
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
     </row>
-    <row r="49" spans="1:14" ht="42.75">
+    <row r="49" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>12</v>
       </c>
@@ -11899,7 +11943,7 @@
       <c r="M49" s="7"/>
       <c r="N49" s="7"/>
     </row>
-    <row r="50" spans="1:14" ht="42.75">
+    <row r="50" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>12</v>
       </c>
@@ -11937,7 +11981,7 @@
       <c r="M50" s="7"/>
       <c r="N50" s="7"/>
     </row>
-    <row r="51" spans="1:14" ht="42.75">
+    <row r="51" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>12</v>
       </c>
@@ -11975,7 +12019,7 @@
       <c r="M51" s="7"/>
       <c r="N51" s="7"/>
     </row>
-    <row r="52" spans="1:14" ht="42.75">
+    <row r="52" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>12</v>
       </c>
@@ -12013,7 +12057,7 @@
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
     </row>
-    <row r="53" spans="1:14" ht="42.75">
+    <row r="53" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>12</v>
       </c>
@@ -12051,7 +12095,7 @@
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
     </row>
-    <row r="54" spans="1:14" ht="42.75">
+    <row r="54" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>12</v>
       </c>
@@ -12089,7 +12133,7 @@
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
     </row>
-    <row r="55" spans="1:14" ht="57">
+    <row r="55" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>12</v>
       </c>
@@ -12127,7 +12171,7 @@
       <c r="M55" s="7"/>
       <c r="N55" s="7"/>
     </row>
-    <row r="56" spans="1:14" ht="57">
+    <row r="56" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>12</v>
       </c>
@@ -12165,7 +12209,7 @@
       <c r="M56" s="7"/>
       <c r="N56" s="7"/>
     </row>
-    <row r="57" spans="1:14" ht="42.75">
+    <row r="57" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
@@ -12203,7 +12247,7 @@
       <c r="M57" s="7"/>
       <c r="N57" s="7"/>
     </row>
-    <row r="58" spans="1:14" ht="42.75">
+    <row r="58" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>12</v>
       </c>
@@ -12241,7 +12285,7 @@
       <c r="M58" s="7"/>
       <c r="N58" s="7"/>
     </row>
-    <row r="59" spans="1:14" ht="57">
+    <row r="59" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>12</v>
       </c>
@@ -12279,7 +12323,7 @@
       <c r="M59" s="7"/>
       <c r="N59" s="7"/>
     </row>
-    <row r="60" spans="1:14" ht="57">
+    <row r="60" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>12</v>
       </c>
@@ -12317,7 +12361,7 @@
       <c r="M60" s="7"/>
       <c r="N60" s="7"/>
     </row>
-    <row r="61" spans="1:14" ht="57">
+    <row r="61" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>12</v>
       </c>
@@ -12355,7 +12399,7 @@
       <c r="M61" s="7"/>
       <c r="N61" s="7"/>
     </row>
-    <row r="62" spans="1:14" ht="57">
+    <row r="62" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>12</v>
       </c>
@@ -12393,7 +12437,7 @@
       <c r="M62" s="7"/>
       <c r="N62" s="7"/>
     </row>
-    <row r="63" spans="1:14" ht="42.75">
+    <row r="63" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>12</v>
       </c>
@@ -12431,7 +12475,7 @@
       <c r="M63" s="7"/>
       <c r="N63" s="7"/>
     </row>
-    <row r="64" spans="1:14" ht="57">
+    <row r="64" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>13</v>
       </c>
@@ -12469,7 +12513,7 @@
       <c r="M64" s="7"/>
       <c r="N64" s="7"/>
     </row>
-    <row r="65" spans="1:14" ht="57">
+    <row r="65" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>13</v>
       </c>
@@ -12507,7 +12551,7 @@
       <c r="M65" s="7"/>
       <c r="N65" s="7"/>
     </row>
-    <row r="66" spans="1:14" ht="57">
+    <row r="66" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>13</v>
       </c>
@@ -12545,7 +12589,7 @@
       <c r="M66" s="7"/>
       <c r="N66" s="7"/>
     </row>
-    <row r="67" spans="1:14" ht="57">
+    <row r="67" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>13</v>
       </c>
@@ -12583,7 +12627,7 @@
       <c r="M67" s="7"/>
       <c r="N67" s="7"/>
     </row>
-    <row r="68" spans="1:14" ht="57">
+    <row r="68" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>13</v>
       </c>
@@ -12621,7 +12665,7 @@
       <c r="M68" s="7"/>
       <c r="N68" s="7"/>
     </row>
-    <row r="69" spans="1:14" ht="57">
+    <row r="69" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>13</v>
       </c>
@@ -12659,7 +12703,7 @@
       <c r="M69" s="7"/>
       <c r="N69" s="7"/>
     </row>
-    <row r="70" spans="1:14" ht="42.75">
+    <row r="70" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>13</v>
       </c>
@@ -12697,7 +12741,7 @@
       <c r="M70" s="7"/>
       <c r="N70" s="7"/>
     </row>
-    <row r="71" spans="1:14" ht="57">
+    <row r="71" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>13</v>
       </c>
@@ -12735,7 +12779,7 @@
       <c r="M71" s="7"/>
       <c r="N71" s="7"/>
     </row>
-    <row r="72" spans="1:14" ht="42.75">
+    <row r="72" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>13</v>
       </c>
@@ -12773,7 +12817,7 @@
       <c r="M72" s="7"/>
       <c r="N72" s="7"/>
     </row>
-    <row r="73" spans="1:14" ht="42.75">
+    <row r="73" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>13</v>
       </c>
@@ -12811,7 +12855,7 @@
       <c r="M73" s="7"/>
       <c r="N73" s="7"/>
     </row>
-    <row r="74" spans="1:14" ht="57">
+    <row r="74" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>13</v>
       </c>
@@ -12849,7 +12893,7 @@
       <c r="M74" s="7"/>
       <c r="N74" s="7"/>
     </row>
-    <row r="75" spans="1:14" ht="42.75">
+    <row r="75" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>13</v>
       </c>
@@ -12887,7 +12931,7 @@
       <c r="M75" s="7"/>
       <c r="N75" s="7"/>
     </row>
-    <row r="76" spans="1:14" ht="57">
+    <row r="76" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>13</v>
       </c>
@@ -12925,7 +12969,7 @@
       <c r="M76" s="7"/>
       <c r="N76" s="7"/>
     </row>
-    <row r="77" spans="1:14" ht="42.75">
+    <row r="77" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>13</v>
       </c>
@@ -12963,7 +13007,7 @@
       <c r="M77" s="7"/>
       <c r="N77" s="7"/>
     </row>
-    <row r="78" spans="1:14" ht="57">
+    <row r="78" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>13</v>
       </c>
@@ -13001,7 +13045,7 @@
       <c r="M78" s="7"/>
       <c r="N78" s="7"/>
     </row>
-    <row r="79" spans="1:14" ht="57">
+    <row r="79" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>13</v>
       </c>
@@ -13039,7 +13083,7 @@
       <c r="M79" s="7"/>
       <c r="N79" s="7"/>
     </row>
-    <row r="80" spans="1:14" ht="42.75">
+    <row r="80" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>13</v>
       </c>
@@ -13077,7 +13121,7 @@
       <c r="M80" s="7"/>
       <c r="N80" s="7"/>
     </row>
-    <row r="81" spans="1:14" ht="42.75">
+    <row r="81" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>13</v>
       </c>
@@ -13115,7 +13159,7 @@
       <c r="M81" s="7"/>
       <c r="N81" s="7"/>
     </row>
-    <row r="82" spans="1:14" ht="42.75">
+    <row r="82" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>13</v>
       </c>
@@ -13153,7 +13197,7 @@
       <c r="M82" s="7"/>
       <c r="N82" s="7"/>
     </row>
-    <row r="83" spans="1:14" ht="42.75">
+    <row r="83" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>13</v>
       </c>
@@ -13191,7 +13235,7 @@
       <c r="M83" s="7"/>
       <c r="N83" s="7"/>
     </row>
-    <row r="84" spans="1:14" ht="42.75">
+    <row r="84" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>14</v>
       </c>
@@ -13229,7 +13273,7 @@
       <c r="M84" s="7"/>
       <c r="N84" s="7"/>
     </row>
-    <row r="85" spans="1:14" ht="42.75">
+    <row r="85" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>14</v>
       </c>
@@ -13267,7 +13311,7 @@
       <c r="M85" s="7"/>
       <c r="N85" s="7"/>
     </row>
-    <row r="86" spans="1:14" ht="42.75">
+    <row r="86" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>14</v>
       </c>
@@ -13305,7 +13349,7 @@
       <c r="M86" s="7"/>
       <c r="N86" s="7"/>
     </row>
-    <row r="87" spans="1:14" ht="42.75">
+    <row r="87" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>14</v>
       </c>
@@ -13343,7 +13387,7 @@
       <c r="M87" s="7"/>
       <c r="N87" s="7"/>
     </row>
-    <row r="88" spans="1:14" ht="42.75">
+    <row r="88" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>14</v>
       </c>
@@ -13381,7 +13425,7 @@
       <c r="M88" s="7"/>
       <c r="N88" s="7"/>
     </row>
-    <row r="89" spans="1:14" ht="42.75">
+    <row r="89" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>14</v>
       </c>
@@ -13419,7 +13463,7 @@
       <c r="M89" s="7"/>
       <c r="N89" s="7"/>
     </row>
-    <row r="90" spans="1:14" ht="42.75">
+    <row r="90" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>14</v>
       </c>
@@ -13457,7 +13501,7 @@
       <c r="M90" s="7"/>
       <c r="N90" s="7"/>
     </row>
-    <row r="91" spans="1:14" ht="42.75">
+    <row r="91" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>14</v>
       </c>
@@ -13495,7 +13539,7 @@
       <c r="M91" s="7"/>
       <c r="N91" s="7"/>
     </row>
-    <row r="92" spans="1:14" ht="42.75">
+    <row r="92" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>14</v>
       </c>
@@ -13533,7 +13577,7 @@
       <c r="M92" s="7"/>
       <c r="N92" s="7"/>
     </row>
-    <row r="93" spans="1:14" ht="42.75">
+    <row r="93" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>14</v>
       </c>
@@ -13571,7 +13615,7 @@
       <c r="M93" s="7"/>
       <c r="N93" s="7"/>
     </row>
-    <row r="94" spans="1:14" ht="42.75">
+    <row r="94" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>14</v>
       </c>
@@ -13609,7 +13653,7 @@
       <c r="M94" s="7"/>
       <c r="N94" s="7"/>
     </row>
-    <row r="95" spans="1:14" ht="57">
+    <row r="95" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>14</v>
       </c>
@@ -13647,7 +13691,7 @@
       <c r="M95" s="7"/>
       <c r="N95" s="7"/>
     </row>
-    <row r="96" spans="1:14" ht="42.75">
+    <row r="96" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>14</v>
       </c>
@@ -13685,7 +13729,7 @@
       <c r="M96" s="7"/>
       <c r="N96" s="7"/>
     </row>
-    <row r="97" spans="1:14" ht="57">
+    <row r="97" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>14</v>
       </c>
@@ -13723,7 +13767,7 @@
       <c r="M97" s="7"/>
       <c r="N97" s="7"/>
     </row>
-    <row r="98" spans="1:14" ht="57">
+    <row r="98" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>14</v>
       </c>
@@ -13761,7 +13805,7 @@
       <c r="M98" s="7"/>
       <c r="N98" s="7"/>
     </row>
-    <row r="99" spans="1:14" ht="42.75">
+    <row r="99" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>15</v>
       </c>
@@ -13799,7 +13843,7 @@
       <c r="M99" s="7"/>
       <c r="N99" s="7"/>
     </row>
-    <row r="100" spans="1:14" ht="42.75">
+    <row r="100" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>15</v>
       </c>
@@ -13837,7 +13881,7 @@
       <c r="M100" s="7"/>
       <c r="N100" s="7"/>
     </row>
-    <row r="101" spans="1:14" ht="57">
+    <row r="101" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>15</v>
       </c>
@@ -13875,7 +13919,7 @@
       <c r="M101" s="7"/>
       <c r="N101" s="7"/>
     </row>
-    <row r="102" spans="1:14" ht="57">
+    <row r="102" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>15</v>
       </c>
@@ -13913,7 +13957,7 @@
       <c r="M102" s="7"/>
       <c r="N102" s="7"/>
     </row>
-    <row r="103" spans="1:14" ht="57">
+    <row r="103" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>15</v>
       </c>
@@ -13951,7 +13995,7 @@
       <c r="M103" s="7"/>
       <c r="N103" s="7"/>
     </row>
-    <row r="104" spans="1:14" ht="57">
+    <row r="104" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>15</v>
       </c>
@@ -13989,7 +14033,7 @@
       <c r="M104" s="7"/>
       <c r="N104" s="7"/>
     </row>
-    <row r="105" spans="1:14" ht="42.75">
+    <row r="105" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>15</v>
       </c>
@@ -14027,7 +14071,7 @@
       <c r="M105" s="7"/>
       <c r="N105" s="7"/>
     </row>
-    <row r="106" spans="1:14" ht="57">
+    <row r="106" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>15</v>
       </c>
@@ -14065,7 +14109,7 @@
       <c r="M106" s="7"/>
       <c r="N106" s="7"/>
     </row>
-    <row r="107" spans="1:14" ht="42.75">
+    <row r="107" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>15</v>
       </c>
@@ -14103,7 +14147,7 @@
       <c r="M107" s="7"/>
       <c r="N107" s="7"/>
     </row>
-    <row r="108" spans="1:14" ht="57">
+    <row r="108" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>15</v>
       </c>
@@ -14141,7 +14185,7 @@
       <c r="M108" s="7"/>
       <c r="N108" s="7"/>
     </row>
-    <row r="109" spans="1:14" ht="57">
+    <row r="109" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>16</v>
       </c>
@@ -14179,7 +14223,7 @@
       <c r="M109" s="7"/>
       <c r="N109" s="7"/>
     </row>
-    <row r="110" spans="1:14" ht="57">
+    <row r="110" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>16</v>
       </c>
@@ -14217,7 +14261,7 @@
       <c r="M110" s="7"/>
       <c r="N110" s="7"/>
     </row>
-    <row r="111" spans="1:14" ht="42.75">
+    <row r="111" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>16</v>
       </c>
@@ -14255,7 +14299,7 @@
       <c r="M111" s="7"/>
       <c r="N111" s="7"/>
     </row>
-    <row r="112" spans="1:14" ht="42.75">
+    <row r="112" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>16</v>
       </c>
@@ -14293,7 +14337,7 @@
       <c r="M112" s="7"/>
       <c r="N112" s="7"/>
     </row>
-    <row r="113" spans="1:14" ht="57">
+    <row r="113" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>16</v>
       </c>
@@ -14331,7 +14375,7 @@
       <c r="M113" s="7"/>
       <c r="N113" s="7"/>
     </row>
-    <row r="114" spans="1:14" ht="57">
+    <row r="114" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>16</v>
       </c>
@@ -14369,7 +14413,7 @@
       <c r="M114" s="7"/>
       <c r="N114" s="7"/>
     </row>
-    <row r="115" spans="1:14" ht="57">
+    <row r="115" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>16</v>
       </c>
@@ -14407,7 +14451,7 @@
       <c r="M115" s="7"/>
       <c r="N115" s="7"/>
     </row>
-    <row r="116" spans="1:14" ht="57">
+    <row r="116" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>16</v>
       </c>
@@ -14445,7 +14489,7 @@
       <c r="M116" s="7"/>
       <c r="N116" s="7"/>
     </row>
-    <row r="117" spans="1:14" ht="42.75">
+    <row r="117" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>16</v>
       </c>
@@ -14483,7 +14527,7 @@
       <c r="M117" s="7"/>
       <c r="N117" s="7"/>
     </row>
-    <row r="118" spans="1:14" ht="42.75">
+    <row r="118" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>16</v>
       </c>
@@ -14521,7 +14565,7 @@
       <c r="M118" s="7"/>
       <c r="N118" s="7"/>
     </row>
-    <row r="119" spans="1:14" ht="42.75">
+    <row r="119" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>17</v>
       </c>
@@ -14559,7 +14603,7 @@
       <c r="M119" s="7"/>
       <c r="N119" s="7"/>
     </row>
-    <row r="120" spans="1:14" ht="42.75">
+    <row r="120" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>17</v>
       </c>
@@ -14597,7 +14641,7 @@
       <c r="M120" s="7"/>
       <c r="N120" s="7"/>
     </row>
-    <row r="121" spans="1:14" ht="42.75">
+    <row r="121" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>17</v>
       </c>
@@ -14635,7 +14679,7 @@
       <c r="M121" s="7"/>
       <c r="N121" s="7"/>
     </row>
-    <row r="122" spans="1:14" ht="42.75">
+    <row r="122" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>17</v>
       </c>
@@ -14673,7 +14717,7 @@
       <c r="M122" s="7"/>
       <c r="N122" s="7"/>
     </row>
-    <row r="123" spans="1:14" ht="42.75">
+    <row r="123" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>17</v>
       </c>
@@ -14711,7 +14755,7 @@
       <c r="M123" s="7"/>
       <c r="N123" s="7"/>
     </row>
-    <row r="124" spans="1:14" ht="42.75">
+    <row r="124" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>17</v>
       </c>
@@ -14749,7 +14793,7 @@
       <c r="M124" s="7"/>
       <c r="N124" s="7"/>
     </row>
-    <row r="125" spans="1:14" ht="42.75">
+    <row r="125" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>17</v>
       </c>
@@ -14787,7 +14831,7 @@
       <c r="M125" s="7"/>
       <c r="N125" s="7"/>
     </row>
-    <row r="126" spans="1:14" ht="42.75">
+    <row r="126" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>17</v>
       </c>
@@ -14825,7 +14869,7 @@
       <c r="M126" s="7"/>
       <c r="N126" s="7"/>
     </row>
-    <row r="127" spans="1:14" ht="42.75">
+    <row r="127" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>17</v>
       </c>
@@ -14863,7 +14907,7 @@
       <c r="M127" s="7"/>
       <c r="N127" s="7"/>
     </row>
-    <row r="128" spans="1:14" ht="42.75">
+    <row r="128" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>17</v>
       </c>
@@ -14901,7 +14945,7 @@
       <c r="M128" s="7"/>
       <c r="N128" s="7"/>
     </row>
-    <row r="129" spans="1:14" ht="42.75">
+    <row r="129" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>18</v>
       </c>
@@ -14939,7 +14983,7 @@
       <c r="M129" s="7"/>
       <c r="N129" s="7"/>
     </row>
-    <row r="130" spans="1:14" ht="42.75">
+    <row r="130" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>18</v>
       </c>
@@ -14977,7 +15021,7 @@
       <c r="M130" s="7"/>
       <c r="N130" s="7"/>
     </row>
-    <row r="131" spans="1:14" ht="42.75">
+    <row r="131" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>18</v>
       </c>
@@ -15015,7 +15059,7 @@
       <c r="M131" s="7"/>
       <c r="N131" s="7"/>
     </row>
-    <row r="132" spans="1:14" ht="42.75">
+    <row r="132" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>18</v>
       </c>
@@ -15053,7 +15097,7 @@
       <c r="M132" s="7"/>
       <c r="N132" s="7"/>
     </row>
-    <row r="133" spans="1:14" ht="45" customHeight="1">
+    <row r="133" spans="1:14" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>18</v>
       </c>
@@ -15091,7 +15135,7 @@
       <c r="M133" s="7"/>
       <c r="N133" s="7"/>
     </row>
-    <row r="134" spans="1:14" ht="28.5">
+    <row r="134" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
         <v>12</v>
       </c>
@@ -15129,7 +15173,7 @@
       <c r="M134" s="7"/>
       <c r="N134" s="7"/>
     </row>
-    <row r="135" spans="1:14" ht="28.5">
+    <row r="135" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>12</v>
       </c>
@@ -15167,7 +15211,7 @@
       <c r="M135" s="7"/>
       <c r="N135" s="7"/>
     </row>
-    <row r="136" spans="1:14" ht="15" customHeight="1">
+    <row r="136" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
         <v>12</v>
       </c>
@@ -15205,7 +15249,7 @@
       <c r="M136" s="7"/>
       <c r="N136" s="7"/>
     </row>
-    <row r="137" spans="1:14" ht="28.5">
+    <row r="137" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
         <v>711</v>
       </c>
@@ -15243,7 +15287,7 @@
       <c r="M137" s="7"/>
       <c r="N137" s="7"/>
     </row>
-    <row r="138" spans="1:14" ht="28.5">
+    <row r="138" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
         <v>711</v>
       </c>
@@ -15281,7 +15325,7 @@
       <c r="M138" s="7"/>
       <c r="N138" s="7"/>
     </row>
-    <row r="139" spans="1:14" ht="28.5">
+    <row r="139" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
         <v>711</v>
       </c>
@@ -15319,7 +15363,7 @@
       <c r="M139" s="7"/>
       <c r="N139" s="7"/>
     </row>
-    <row r="140" spans="1:14" ht="15" customHeight="1">
+    <row r="140" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="7" t="s">
         <v>711</v>
       </c>
@@ -15357,7 +15401,7 @@
       <c r="M140" s="7"/>
       <c r="N140" s="7"/>
     </row>
-    <row r="141" spans="1:14" ht="28.5">
+    <row r="141" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
         <v>5</v>
       </c>
@@ -15395,7 +15439,7 @@
       <c r="M141" s="7"/>
       <c r="N141" s="7"/>
     </row>
-    <row r="142" spans="1:14" ht="15" customHeight="1">
+    <row r="142" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="7" t="s">
         <v>5</v>
       </c>
@@ -15433,7 +15477,7 @@
       <c r="M142" s="7"/>
       <c r="N142" s="7"/>
     </row>
-    <row r="143" spans="1:14" ht="28.5">
+    <row r="143" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>5</v>
       </c>
@@ -15471,7 +15515,7 @@
       <c r="M143" s="7"/>
       <c r="N143" s="7"/>
     </row>
-    <row r="144" spans="1:14" ht="75" customHeight="1">
+    <row r="144" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="7" t="s">
         <v>6</v>
       </c>
@@ -15509,7 +15553,7 @@
       <c r="M144" s="7"/>
       <c r="N144" s="7"/>
     </row>
-    <row r="145" spans="1:14" ht="15" customHeight="1">
+    <row r="145" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
         <v>6</v>
       </c>
@@ -15547,7 +15591,7 @@
       <c r="M145" s="7"/>
       <c r="N145" s="7"/>
     </row>
-    <row r="146" spans="1:14" ht="15" customHeight="1">
+    <row r="146" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="7" t="s">
         <v>6</v>
       </c>
@@ -15585,7 +15629,7 @@
       <c r="M146" s="7"/>
       <c r="N146" s="7"/>
     </row>
-    <row r="147" spans="1:14" ht="28.5">
+    <row r="147" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
         <v>6</v>
       </c>
@@ -15623,7 +15667,7 @@
       <c r="M147" s="7"/>
       <c r="N147" s="7"/>
     </row>
-    <row r="148" spans="1:14" ht="28.5">
+    <row r="148" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A148" s="7" t="s">
         <v>770</v>
       </c>
@@ -15661,7 +15705,7 @@
       <c r="M148" s="7"/>
       <c r="N148" s="7"/>
     </row>
-    <row r="149" spans="1:14" ht="15" customHeight="1">
+    <row r="149" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
         <v>770</v>
       </c>
@@ -15699,7 +15743,7 @@
       <c r="M149" s="7"/>
       <c r="N149" s="7"/>
     </row>
-    <row r="150" spans="1:14" ht="28.5">
+    <row r="150" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A150" s="7" t="s">
         <v>781</v>
       </c>
@@ -15737,7 +15781,7 @@
       <c r="M150" s="7"/>
       <c r="N150" s="7"/>
     </row>
-    <row r="151" spans="1:14" ht="28.5">
+    <row r="151" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
         <v>781</v>
       </c>
@@ -15775,7 +15819,7 @@
       <c r="M151" s="7"/>
       <c r="N151" s="7"/>
     </row>
-    <row r="152" spans="1:14" ht="15" customHeight="1">
+    <row r="152" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="7" t="s">
         <v>793</v>
       </c>
@@ -15813,7 +15857,7 @@
       <c r="M152" s="7"/>
       <c r="N152" s="7"/>
     </row>
-    <row r="153" spans="1:14" ht="15" customHeight="1">
+    <row r="153" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
         <v>793</v>
       </c>
@@ -15851,7 +15895,7 @@
       <c r="M153" s="7"/>
       <c r="N153" s="7"/>
     </row>
-    <row r="154" spans="1:14" ht="15" customHeight="1">
+    <row r="154" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="7" t="s">
         <v>812</v>
       </c>
@@ -15889,7 +15933,7 @@
       <c r="M154" s="7"/>
       <c r="N154" s="7"/>
     </row>
-    <row r="155" spans="1:14" ht="28.5">
+    <row r="155" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A155" s="7" t="s">
         <v>818</v>
       </c>
@@ -15927,7 +15971,7 @@
       <c r="M155" s="7"/>
       <c r="N155" s="7"/>
     </row>
-    <row r="156" spans="1:14" ht="15" customHeight="1">
+    <row r="156" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="7" t="s">
         <v>824</v>
       </c>
@@ -15963,7 +16007,7 @@
       <c r="M156" s="7"/>
       <c r="N156" s="7"/>
     </row>
-    <row r="157" spans="1:14" ht="42.75">
+    <row r="157" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A157" s="7" t="s">
         <v>829</v>
       </c>
@@ -15999,7 +16043,7 @@
       <c r="M157" s="7"/>
       <c r="N157" s="7"/>
     </row>
-    <row r="158" spans="1:14" ht="28.5">
+    <row r="158" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A158" s="7" t="s">
         <v>834</v>
       </c>
@@ -16037,7 +16081,7 @@
       <c r="M158" s="7"/>
       <c r="N158" s="7"/>
     </row>
-    <row r="159" spans="1:14" ht="15" customHeight="1">
+    <row r="159" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
         <v>840</v>
       </c>
@@ -16073,7 +16117,7 @@
       <c r="M159" s="7"/>
       <c r="N159" s="7"/>
     </row>
-    <row r="160" spans="1:14" ht="42.75">
+    <row r="160" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
         <v>12</v>
       </c>
@@ -16111,39 +16155,79 @@
       <c r="M160" s="7"/>
       <c r="N160" s="7"/>
     </row>
-    <row r="161" spans="1:14" ht="15" customHeight="1">
-      <c r="A161" s="7"/>
-      <c r="B161" s="7"/>
-      <c r="C161" s="7"/>
-      <c r="D161" s="7"/>
-      <c r="E161" s="7"/>
-      <c r="F161" s="7"/>
+    <row r="161" spans="1:14" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="7" t="s">
+        <v>829</v>
+      </c>
+      <c r="B161" s="7" t="s">
+        <v>865</v>
+      </c>
+      <c r="C161" s="7" t="s">
+        <v>867</v>
+      </c>
+      <c r="D161" s="7" t="s">
+        <v>869</v>
+      </c>
+      <c r="E161" s="7" t="s">
+        <v>870</v>
+      </c>
+      <c r="F161" s="7" t="s">
+        <v>872</v>
+      </c>
       <c r="G161" s="7"/>
-      <c r="H161" s="7"/>
+      <c r="H161" s="7" t="s">
+        <v>874</v>
+      </c>
       <c r="I161" s="7"/>
-      <c r="J161" s="3"/>
-      <c r="K161" s="3"/>
-      <c r="L161" s="7"/>
+      <c r="J161" s="6">
+        <v>45957</v>
+      </c>
+      <c r="K161" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L161" s="10" t="s">
+        <v>35</v>
+      </c>
       <c r="M161" s="7"/>
       <c r="N161" s="7"/>
     </row>
-    <row r="162" spans="1:14">
-      <c r="A162" s="7"/>
-      <c r="B162" s="7"/>
-      <c r="C162" s="7"/>
-      <c r="D162" s="7"/>
-      <c r="E162" s="7"/>
-      <c r="F162" s="7"/>
+    <row r="162" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A162" s="7" t="s">
+        <v>829</v>
+      </c>
+      <c r="B162" s="7" t="s">
+        <v>866</v>
+      </c>
+      <c r="C162" s="7" t="s">
+        <v>868</v>
+      </c>
+      <c r="D162" s="7" t="s">
+        <v>869</v>
+      </c>
+      <c r="E162" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="F162" s="7" t="s">
+        <v>873</v>
+      </c>
       <c r="G162" s="7"/>
-      <c r="H162" s="7"/>
+      <c r="H162" s="7" t="s">
+        <v>875</v>
+      </c>
       <c r="I162" s="7"/>
-      <c r="J162" s="3"/>
-      <c r="K162" s="3"/>
-      <c r="L162" s="7"/>
+      <c r="J162" s="6">
+        <v>45957</v>
+      </c>
+      <c r="K162" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L162" s="10" t="s">
+        <v>35</v>
+      </c>
       <c r="M162" s="7"/>
       <c r="N162" s="7"/>
     </row>
-    <row r="163" spans="1:14" ht="15" customHeight="1">
+    <row r="163" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="7"/>
       <c r="B163" s="7"/>
       <c r="C163" s="7"/>
@@ -16159,7 +16243,7 @@
       <c r="M163" s="7"/>
       <c r="N163" s="7"/>
     </row>
-    <row r="164" spans="1:14">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="7"/>
       <c r="B164" s="7"/>
       <c r="C164" s="7"/>
@@ -16175,7 +16259,7 @@
       <c r="M164" s="7"/>
       <c r="N164" s="7"/>
     </row>
-    <row r="165" spans="1:14">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="7"/>
       <c r="B165" s="7"/>
       <c r="C165" s="7"/>
@@ -16191,7 +16275,7 @@
       <c r="M165" s="7"/>
       <c r="N165" s="7"/>
     </row>
-    <row r="166" spans="1:14" ht="15" customHeight="1">
+    <row r="166" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="7"/>
       <c r="B166" s="7"/>
       <c r="C166" s="7"/>
@@ -16207,7 +16291,7 @@
       <c r="M166" s="7"/>
       <c r="N166" s="7"/>
     </row>
-    <row r="167" spans="1:14">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B167" s="7"/>
       <c r="C167" s="7"/>
       <c r="D167" s="7"/>
@@ -16222,7 +16306,7 @@
       <c r="M167" s="7"/>
       <c r="N167" s="7"/>
     </row>
-    <row r="168" spans="1:14" ht="30" customHeight="1">
+    <row r="168" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B168" s="7"/>
       <c r="C168" s="7"/>
       <c r="D168" s="7"/>
@@ -16237,7 +16321,7 @@
       <c r="M168" s="7"/>
       <c r="N168" s="7"/>
     </row>
-    <row r="169" spans="1:14">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B169" s="7"/>
       <c r="C169" s="7"/>
       <c r="D169" s="7"/>
@@ -16252,7 +16336,7 @@
       <c r="M169" s="7"/>
       <c r="N169" s="7"/>
     </row>
-    <row r="170" spans="1:14" ht="15" customHeight="1">
+    <row r="170" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B170" s="7"/>
       <c r="C170" s="7"/>
       <c r="D170" s="7"/>
@@ -16269,7 +16353,7 @@
       </c>
       <c r="N170" s="7"/>
     </row>
-    <row r="171" spans="1:14">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B171" s="7"/>
       <c r="C171" s="7"/>
       <c r="D171" s="7"/>
@@ -16284,7 +16368,7 @@
       <c r="M171" s="7"/>
       <c r="N171" s="7"/>
     </row>
-    <row r="172" spans="1:14" ht="30" customHeight="1">
+    <row r="172" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B172" s="7"/>
       <c r="C172" s="7"/>
       <c r="D172" s="7"/>
@@ -16299,7 +16383,7 @@
       <c r="M172" s="7"/>
       <c r="N172" s="7"/>
     </row>
-    <row r="173" spans="1:14">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B173" s="7"/>
       <c r="C173" s="7"/>
       <c r="D173" s="7"/>
@@ -16312,7 +16396,7 @@
       <c r="K173" s="3"/>
       <c r="L173" s="7"/>
     </row>
-    <row r="174" spans="1:14">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B174" s="7"/>
       <c r="C174" s="7"/>
       <c r="D174" s="7"/>
@@ -16325,7 +16409,7 @@
       <c r="K174" s="3"/>
       <c r="L174" s="7"/>
     </row>
-    <row r="175" spans="1:14">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B175" s="7"/>
       <c r="C175" s="7"/>
       <c r="D175" s="7"/>
@@ -16338,7 +16422,7 @@
       <c r="K175" s="3"/>
       <c r="L175" s="7"/>
     </row>
-    <row r="176" spans="1:14">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B176" s="7"/>
       <c r="C176" s="7"/>
       <c r="D176" s="7"/>
@@ -16351,7 +16435,7 @@
       <c r="K176" s="3"/>
       <c r="L176" s="7"/>
     </row>
-    <row r="177" spans="2:12">
+    <row r="177" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B177" s="7"/>
       <c r="C177" s="7"/>
       <c r="D177" s="7"/>
@@ -16364,7 +16448,7 @@
       <c r="K177" s="3"/>
       <c r="L177" s="7"/>
     </row>
-    <row r="178" spans="2:12">
+    <row r="178" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B178" s="7"/>
       <c r="C178" s="7"/>
       <c r="D178" s="7"/>
@@ -16377,7 +16461,7 @@
       <c r="K178" s="3"/>
       <c r="L178" s="7"/>
     </row>
-    <row r="179" spans="2:12">
+    <row r="179" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B179" s="7"/>
       <c r="C179" s="7"/>
       <c r="D179" s="7"/>
@@ -16390,7 +16474,7 @@
       <c r="K179" s="3"/>
       <c r="L179" s="7"/>
     </row>
-    <row r="180" spans="2:12">
+    <row r="180" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B180" s="7"/>
       <c r="C180" s="7"/>
       <c r="D180" s="7"/>
@@ -16403,7 +16487,7 @@
       <c r="K180" s="3"/>
       <c r="L180" s="7"/>
     </row>
-    <row r="181" spans="2:12">
+    <row r="181" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B181" s="7"/>
       <c r="C181" s="7"/>
       <c r="D181" s="7"/>
@@ -16416,7 +16500,7 @@
       <c r="K181" s="3"/>
       <c r="L181" s="7"/>
     </row>
-    <row r="182" spans="2:12">
+    <row r="182" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B182" s="7"/>
       <c r="C182" s="7"/>
       <c r="D182" s="7"/>
@@ -16429,7 +16513,7 @@
       <c r="K182" s="3"/>
       <c r="L182" s="7"/>
     </row>
-    <row r="183" spans="2:12">
+    <row r="183" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B183" s="7"/>
       <c r="C183" s="7"/>
       <c r="D183" s="7"/>
@@ -16442,7 +16526,7 @@
       <c r="K183" s="3"/>
       <c r="L183" s="7"/>
     </row>
-    <row r="184" spans="2:12">
+    <row r="184" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
       <c r="D184" s="7"/>
@@ -16458,32 +16542,32 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="L4:L153">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"PENDING"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>"PASS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
       <formula>"FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L161:L165 K164 L167:L184">
-    <cfRule type="cellIs" dxfId="2" priority="34" operator="equal">
+  <conditionalFormatting sqref="L163:L165 K164 L167:L184">
+    <cfRule type="cellIs" dxfId="14" priority="34" operator="equal">
       <formula>"PENDING"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="35" operator="equal">
       <formula>"PASS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="36" operator="equal">
       <formula>"FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L167:L184 K164 L161:L165 L4:L153" xr:uid="{1E8D2D6D-4EE7-40E2-A622-3458BDCF08AD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L167:L184 K164 L4:L153 L163:L165" xr:uid="{1E8D2D6D-4EE7-40E2-A622-3458BDCF08AD}">
       <formula1>"PASS,PENDING,FAIL"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A161:A166 A4:A153" xr:uid="{F4675041-A1B8-4B65-822E-23AD6AB864A0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A4:A153 A163:A166" xr:uid="{F4675041-A1B8-4B65-822E-23AD6AB864A0}">
       <formula1>INDIRECT("Modulos[MODULOS]")</formula1>
     </dataValidation>
   </dataValidations>
@@ -16500,25 +16584,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58476477-5BDE-4E9D-BCDF-FD6E3C12EE95}">
   <dimension ref="A2:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.125" customWidth="1"/>
-    <col min="9" max="9" width="24.75" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.375" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.140625" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="23.25" customHeight="1">
+    <row r="2" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>805</v>
       </c>
@@ -16529,7 +16613,7 @@
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>807</v>
       </c>
@@ -16546,7 +16630,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>809</v>
       </c>
@@ -16559,7 +16643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -16572,7 +16656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="21.75" customHeight="1">
+    <row r="6" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -16585,7 +16669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -16598,7 +16682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>808</v>
       </c>
@@ -16615,7 +16699,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="28.5">
+    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>807</v>
       </c>
@@ -16623,7 +16707,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>116</v>
       </c>
@@ -16631,7 +16715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
@@ -16639,7 +16723,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>132</v>
       </c>
@@ -16647,7 +16731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>808</v>
       </c>
@@ -16664,7 +16748,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B55000D3-4297-437F-A419-CEB79EC3F6C0}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16672,6 +16756,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E158E2AB9B4F924688B558FA982B40CF" ma:contentTypeVersion="3" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ce5f689dcf51305603cb0d070870d6dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="def3e2b2-904e-4359-b966-59b7b32cd06e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="252587ffdfea7067e66d630466c44dd6" ns2:_="">
     <xsd:import namespace="def3e2b2-904e-4359-b966-59b7b32cd06e"/>
@@ -16809,22 +16908,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CABA5C2-04D8-4DC5-BBFB-FF9AC004B268}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A2950B-6D37-4A45-BCA2-DEBA33559D5B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1F0EA96-F162-49AF-B0BE-A54883795866}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16840,21 +16941,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A2950B-6D37-4A45-BCA2-DEBA33559D5B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CABA5C2-04D8-4DC5-BBFB-FF9AC004B268}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>